<commit_message>
Completed OAH org for orders-deselected-waving DB Alert
</commit_message>
<xml_diff>
--- a/lia-pack-uom/WarehouseDetail_records copy(Lia-pack-uom).xlsx
+++ b/lia-pack-uom/WarehouseDetail_records copy(Lia-pack-uom).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rndc/Desktop/Work related/Documents/lia-pack-uom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C01F6E1B-AE8C-634C-A4D3-131CFB6D951E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E076FB-2BA6-584F-B7D7-7E6535886822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="1240" windowWidth="19220" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF01000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF01000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Actual warehouselocationdetail " sheetId="7" r:id="rId1"/>
@@ -2760,7 +2760,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -2794,7 +2794,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3137,7 +3136,7 @@
     <col min="3" max="3" width="12.6640625" customWidth="1"/>
     <col min="4" max="4" width="17.5" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="25.5" style="17" customWidth="1"/>
+    <col min="6" max="6" width="25.5" customWidth="1"/>
     <col min="7" max="7" width="8" customWidth="1"/>
     <col min="8" max="8" width="7.1640625" customWidth="1"/>
     <col min="9" max="9" width="6.83203125" customWidth="1"/>
@@ -3160,7 +3159,7 @@
       <c r="E1" t="s">
         <v>233</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" t="s">
         <v>122</v>
       </c>
       <c r="G1" t="s">
@@ -3192,7 +3191,7 @@
       <c r="E2">
         <v>31</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" t="s">
         <v>238</v>
       </c>
       <c r="G2" t="s">
@@ -3224,7 +3223,7 @@
       <c r="E3">
         <v>31</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" t="s">
         <v>123</v>
       </c>
       <c r="G3" t="s">
@@ -3256,7 +3255,7 @@
       <c r="E4">
         <v>31</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" t="s">
         <v>123</v>
       </c>
       <c r="G4" t="s">
@@ -3288,7 +3287,7 @@
       <c r="E5">
         <v>31</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" t="s">
         <v>123</v>
       </c>
       <c r="G5" t="s">
@@ -3320,7 +3319,7 @@
       <c r="E6">
         <v>31</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" t="s">
         <v>123</v>
       </c>
       <c r="G6" t="s">
@@ -3352,7 +3351,7 @@
       <c r="E7">
         <v>31</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" t="s">
         <v>123</v>
       </c>
       <c r="G7" t="s">
@@ -3384,7 +3383,7 @@
       <c r="E8">
         <v>31</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F8" t="s">
         <v>123</v>
       </c>
       <c r="G8" t="s">
@@ -3416,7 +3415,7 @@
       <c r="E9">
         <v>31</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" t="s">
         <v>123</v>
       </c>
       <c r="G9" t="s">
@@ -3448,7 +3447,7 @@
       <c r="E10">
         <v>31</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="F10" t="s">
         <v>123</v>
       </c>
       <c r="G10" t="s">
@@ -3480,7 +3479,7 @@
       <c r="E11">
         <v>31</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" t="s">
         <v>240</v>
       </c>
       <c r="G11" t="s">
@@ -3512,7 +3511,7 @@
       <c r="E12">
         <v>31</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="F12" t="s">
         <v>123</v>
       </c>
       <c r="G12" t="s">
@@ -3544,7 +3543,7 @@
       <c r="E13">
         <v>31</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" t="s">
         <v>123</v>
       </c>
       <c r="G13" t="s">
@@ -3576,7 +3575,7 @@
       <c r="E14">
         <v>31</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" t="s">
         <v>123</v>
       </c>
       <c r="G14" t="s">
@@ -3608,7 +3607,7 @@
       <c r="E15">
         <v>31</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" t="s">
         <v>241</v>
       </c>
       <c r="G15" t="s">
@@ -3640,7 +3639,7 @@
       <c r="E16">
         <v>31</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" t="s">
         <v>123</v>
       </c>
       <c r="G16" t="s">
@@ -3672,7 +3671,7 @@
       <c r="E17">
         <v>31</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" t="s">
         <v>123</v>
       </c>
       <c r="G17" t="s">
@@ -3704,7 +3703,7 @@
       <c r="E18">
         <v>31</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" t="s">
         <v>123</v>
       </c>
       <c r="G18" t="s">
@@ -3736,7 +3735,7 @@
       <c r="E19">
         <v>31</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" t="s">
         <v>123</v>
       </c>
       <c r="G19" t="s">
@@ -3768,7 +3767,7 @@
       <c r="E20">
         <v>31</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" t="s">
         <v>123</v>
       </c>
       <c r="G20" t="s">
@@ -3800,7 +3799,7 @@
       <c r="E21">
         <v>31</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="F21" t="s">
         <v>123</v>
       </c>
       <c r="G21" t="s">
@@ -3832,7 +3831,7 @@
       <c r="E22">
         <v>31</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" t="s">
         <v>123</v>
       </c>
       <c r="G22" t="s">
@@ -3864,7 +3863,7 @@
       <c r="E23">
         <v>31</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F23" t="s">
         <v>123</v>
       </c>
       <c r="G23" t="s">
@@ -3896,7 +3895,7 @@
       <c r="E24">
         <v>31</v>
       </c>
-      <c r="F24" s="17" t="s">
+      <c r="F24" t="s">
         <v>123</v>
       </c>
       <c r="G24" t="s">
@@ -3928,7 +3927,7 @@
       <c r="E25">
         <v>31</v>
       </c>
-      <c r="F25" s="17" t="s">
+      <c r="F25" t="s">
         <v>123</v>
       </c>
       <c r="G25" t="s">
@@ -3960,7 +3959,7 @@
       <c r="E26">
         <v>31</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="F26" t="s">
         <v>242</v>
       </c>
       <c r="G26" t="s">
@@ -3992,7 +3991,7 @@
       <c r="E27">
         <v>31</v>
       </c>
-      <c r="F27" s="17" t="s">
+      <c r="F27" t="s">
         <v>123</v>
       </c>
       <c r="G27" t="s">
@@ -4024,7 +4023,7 @@
       <c r="E28">
         <v>31</v>
       </c>
-      <c r="F28" s="17" t="s">
+      <c r="F28" t="s">
         <v>123</v>
       </c>
       <c r="G28" t="s">
@@ -4056,7 +4055,7 @@
       <c r="E29">
         <v>31</v>
       </c>
-      <c r="F29" s="17" t="s">
+      <c r="F29" t="s">
         <v>123</v>
       </c>
       <c r="G29" t="s">
@@ -4088,7 +4087,7 @@
       <c r="E30">
         <v>31</v>
       </c>
-      <c r="F30" s="17" t="s">
+      <c r="F30" t="s">
         <v>243</v>
       </c>
       <c r="G30" t="s">
@@ -4120,7 +4119,7 @@
       <c r="E31">
         <v>31</v>
       </c>
-      <c r="F31" s="17" t="s">
+      <c r="F31" t="s">
         <v>123</v>
       </c>
       <c r="G31" t="s">
@@ -4152,7 +4151,7 @@
       <c r="E32">
         <v>31</v>
       </c>
-      <c r="F32" s="17" t="s">
+      <c r="F32" t="s">
         <v>123</v>
       </c>
       <c r="G32" t="s">
@@ -4184,7 +4183,7 @@
       <c r="E33">
         <v>31</v>
       </c>
-      <c r="F33" s="17" t="s">
+      <c r="F33" t="s">
         <v>123</v>
       </c>
       <c r="G33" t="s">
@@ -4216,7 +4215,7 @@
       <c r="E34">
         <v>31</v>
       </c>
-      <c r="F34" s="17" t="s">
+      <c r="F34" t="s">
         <v>123</v>
       </c>
       <c r="G34" t="s">
@@ -4248,7 +4247,7 @@
       <c r="E35">
         <v>31</v>
       </c>
-      <c r="F35" s="17" t="s">
+      <c r="F35" t="s">
         <v>123</v>
       </c>
       <c r="G35" t="s">
@@ -4280,7 +4279,7 @@
       <c r="E36">
         <v>31</v>
       </c>
-      <c r="F36" s="17" t="s">
+      <c r="F36" t="s">
         <v>123</v>
       </c>
       <c r="G36" t="s">
@@ -4312,7 +4311,7 @@
       <c r="E37">
         <v>31</v>
       </c>
-      <c r="F37" s="17" t="s">
+      <c r="F37" t="s">
         <v>123</v>
       </c>
       <c r="G37" t="s">
@@ -4344,7 +4343,7 @@
       <c r="E38">
         <v>31</v>
       </c>
-      <c r="F38" s="17" t="s">
+      <c r="F38" t="s">
         <v>123</v>
       </c>
       <c r="G38" t="s">
@@ -4376,7 +4375,7 @@
       <c r="E39">
         <v>31</v>
       </c>
-      <c r="F39" s="17" t="s">
+      <c r="F39" t="s">
         <v>123</v>
       </c>
       <c r="G39" t="s">
@@ -4408,7 +4407,7 @@
       <c r="E40">
         <v>31</v>
       </c>
-      <c r="F40" s="17" t="s">
+      <c r="F40" t="s">
         <v>123</v>
       </c>
       <c r="G40" t="s">
@@ -4440,7 +4439,7 @@
       <c r="E41">
         <v>31</v>
       </c>
-      <c r="F41" s="17" t="s">
+      <c r="F41" t="s">
         <v>123</v>
       </c>
       <c r="G41" t="s">
@@ -4472,7 +4471,7 @@
       <c r="E42">
         <v>31</v>
       </c>
-      <c r="F42" s="17" t="s">
+      <c r="F42" t="s">
         <v>244</v>
       </c>
       <c r="G42" t="s">
@@ -4504,7 +4503,7 @@
       <c r="E43">
         <v>31</v>
       </c>
-      <c r="F43" s="17" t="s">
+      <c r="F43" t="s">
         <v>123</v>
       </c>
       <c r="G43" t="s">
@@ -4536,7 +4535,7 @@
       <c r="E44">
         <v>31</v>
       </c>
-      <c r="F44" s="17" t="s">
+      <c r="F44" t="s">
         <v>123</v>
       </c>
       <c r="G44" t="s">

</xml_diff>

<commit_message>
Created update-ccEmail-payload.sql for lia-pack-uom and order-stuck-15m
</commit_message>
<xml_diff>
--- a/lia-pack-uom/WarehouseDetail_records copy(Lia-pack-uom).xlsx
+++ b/lia-pack-uom/WarehouseDetail_records copy(Lia-pack-uom).xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rndc/Desktop/Work related/Documents/lia-pack-uom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E076FB-2BA6-584F-B7D7-7E6535886822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC4A733-F269-2B42-A0A9-270EEBB7E6FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF01000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF01000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Actual warehouselocationdetail " sheetId="7" r:id="rId1"/>
-    <sheet name="After_remaining_03_02_updates" sheetId="6" r:id="rId2"/>
+    <sheet name="After_remaining_03_23_updates" sheetId="6" r:id="rId2"/>
     <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
     <sheet name="Before_03_02_updates" sheetId="5" r:id="rId4"/>
     <sheet name="warehouselocation" sheetId="2" r:id="rId5"/>
@@ -22,7 +22,7 @@
     <sheet name="Sheet2" sheetId="4" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">After_remaining_03_02_updates!$A$1:$K$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">After_remaining_03_23_updates!$A$1:$K$47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Before_03_02_updates!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Sheet1!$B$69:$I$69</definedName>
   </definedNames>
@@ -2592,33 +2592,6 @@
 }</t>
   </si>
   <si>
-    <t>Null</t>
-  </si>
-  <si>
-    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"LOU","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://10.248.248.195:3306/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for '$orgId$ + $dataSource$ + $alertName$' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"noreply@rndc-usa.com","toEmail":"frankie.troncosa@rndc-usa.com,erik.thoreson@rndc-usa.com,chadd.vankampen@rndc-usa.com, michael.gallagher@rndc-usa.com, wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
-  </si>
-  <si>
-    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"PEN","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://10.248.248.195:3306/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for '$orgId$ + $dataSource$ + $alertName$' was triggered.","fromEmail":"noreply@rndc-usa.com","toEmail":"Ryan.Metz@rndc-usa.com, John.Hall@rndc-usa.com, Anthony.Coleman@rndc-usa.com, Dazzle.Keyser@rndc-usa.com, Douglas.Garner@rndc-usa.com, wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
-  </si>
-  <si>
-    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"POR","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://10.248.248.195:3306/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for '$orgId$ + $dataSource$ + $alertName$' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"noreply@rndc-usa.com","toEmail":"wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM, DL_MANH_RNDC_MAWM_PSO@manh.com, DL_RNDC_MAWM_CSO@manh.com, wmsinternal@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
-  </si>
-  <si>
-    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"ARK","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://10.248.248.195:3306/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for '$orgId$ + $dataSource$ + $alertName$' was triggered. ***MSP TO CLEAN UP***","fromEmail":"noreply@rndc-usa.com","toEmail":"Kim.Crawford@rndc-usa.com, Joe.Thompson@rndc-usa.com, Joshua.Edens@rndc-usa.com, wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
-  </si>
-  <si>
-    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"ASH","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://10.248.248.195:3306/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for '$orgId$ + $dataSource$ + $alertName$' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"noreply@rndc-usa.com","toEmail":"Jonathan.Snell@RNDC-USA.COM, Preston.Mccauley@RNDC-USA.COM, Rob.Garcia@RNDC-USA.COM, Jordan.Stoll@rndc-usa.com, Kerry.Partridge@RNDC-USA.COM, Richard.Gay@RNDC-USA.COM, Billy.Calloway@RNDC-USA.COM, Ryan.Black@rndc-usa.com, wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
-  </si>
-  <si>
-    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"RVR","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://10.248.248.195:3306/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for '$orgId$ + $dataSource$ + $alertName$' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"noreply@rndc-usa.com","toEmail":"wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM, DL_MANH_RNDC_MAWM_PSO@manh.com, DL_RNDC_MAWM_CSO@manh.com, wmsinternal@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table","csv"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
-  </si>
-  <si>
-    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"CHI","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://10.248.248.195:3306/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for '$orgId$ + $dataSource$ + $alertName$' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"noreply@rndc-usa.com","toEmail":"wmsinternal@RNDC-USA.COM, WMSConsultant@RNDC-USA.COM, wmsmspsupport@rndc-usa.com,wmsinternal@RNDC-USA.COM, DL_MANH_RNDC_MAWM_PSO@manh.com, DL_RNDC_MAWM_CSO@manh.com,CHIAutomationSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table","csv"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
-  </si>
-  <si>
-    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"ATL","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://10.248.248.195:3306/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for '$orgId$ + $dataSource$ + $alertName$' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"noreply@rndc-usa.com","toEmail":"Jennifer.Arrington@RNDC-USA.COM, Steven.Pacheco@RNDC-USA.COM, AJ.Jones@RNDC-USA.COM, Cody.Byars@RNDC-USA.COM, Patrick.Guyton@RNDC-USA.COM,Taylor.Kratzer@rndc-usa.com, Juan.gutierrez@rndc-usa.com,Raymond.Tuff@RNDC-USA.COM, wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}</t>
-  </si>
-  <si>
     <t>warehousedetailid</t>
   </si>
   <si>
@@ -2662,6 +2635,33 @@
   </si>
   <si>
     <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"LOU","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://10.248.248.195:3306/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for '$orgId$ + $dataSource$ + $alertName$' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"noreply@rndc-usa.com","toEmail":"frankie.troncosa@rndc-usa.com,erik.thoreson@rndc-usa.com,chadd.vankampen@rndc-usa.com, michael.gallagher@rndc-usa.com, wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}</t>
+  </si>
+  <si>
+    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"PEN","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://{host}:{port}/{schema}"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for ''$orgId$ + $dataSource$ + $alertName$'' was triggered.","fromEmail":"wms-tools-no-reply@rndc-usa.com","toEmail":"Ryan.Metz@rndc-usa.com, John.Hall@rndc-usa.com, Anthony.Coleman@rndc-usa.com, Dazzle.Keyser@rndc-usa.com, Douglas.Garner@rndc-usa.com", "ccEmail": "wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
+  </si>
+  <si>
+    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"POR","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://{host}:{port}/{schema}"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for ''$orgId$ + $dataSource$ + $alertName$'' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"wms-tools-no-reply@rndc-usa.com","toEmail":"wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM, DL_MANH_RNDC_MAWM_PSO@manh.com, DL_RNDC_MAWM_CSO@manh.com, wmsinternal@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
+  </si>
+  <si>
+    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"ARK","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://{host}:{port}/{schema}"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for ''$orgId$ + $dataSource$ + $alertName$'' was triggered. ***MSP TO CLEAN UP***","fromEmail":"wms-tools-no-reply@rndc-usa.com","toEmail":"Kim.Crawford@rndc-usa.com, Joe.Thompson@rndc-usa.com, Joshua.Edens@rndc-usa.com", "ccEmail": "wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
+  </si>
+  <si>
+    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","orgId":"LOU","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:mysql://{host}:{port}/{schema}"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for ''$orgId$ + $dataSource$ + $alertName$'' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"wms-tools-no-reply@rndc-usa.com","toEmail":"frankie.troncosa@rndc-usa.com,erik.thoreson@rndc-usa.com,chadd.vankampen@rndc-usa.com, michael.gallagher@rndc-usa.com", "ccEmail": "wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
+  </si>
+  <si>
+    <t>(named, but disabled and no payload entry in warehouselocationdetail)</t>
+  </si>
+  <si>
+    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for ''$orgId$ + $dataSource$ + $alertName$'' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"wms-tools-no-reply@rndc-usa.com","toEmail": "Jonathan.Snell@RNDC-USA.COM, Preston.Mccauley@RNDC-USA.COM, Rob.Garcia@RNDC-USA.COM, Jordan.Stoll@rndc-usa.com, Kerry.Partridge@RNDC-USA.COM, Richard.Gay@RNDC-USA.COM, Billy.Calloway@RNDC-USA.COM, Ryan.Black@rndc-usa.com", "ccEmail": "wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
+  </si>
+  <si>
+    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for ''$orgId$ + $dataSource$ + $alertName$'' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"wms-tools-no-reply@rndc-usa.com","toEmail": "Jennifer.Arrington@RNDC-USA.COM, Steven.Pacheco@RNDC-USA.COM, AJ.Jones@RNDC-USA.COM, Cody.Byars@RNDC-USA.COM, Patrick.Guyton@RNDC-USA.COM,Taylor.Kratzer@rndc-usa.com, Juan.gutierrez@rndc-usa.com,Raymond.Tuff@RNDC-USA.COM", "ccEmail": "wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
+  </si>
+  <si>
+    <t>{"alertName":"LIA RECORDS WITH PACK UOM TYPE POPULATED","dataSource":"MAWM","database":{"connection":"MAPRD_NEW","type":"MySQL","uri":"jdbc:{host}:{port}/information_schema"},"email":{"subject":"Splunk Alert: $orgId$ + $dataSource$ + $alertName$","body":"The alert condition for ''$orgId$ + $dataSource$ + $alertName$'' was triggered.***MSP TO CLEAN UP*** Clear the PACK UOM TYPE ID and PACK UOM QUANTITY from the Location Item Assignment UI.","fromEmail":"wms-tools-no-reply@rndc-usa.com","toEmail":"wmsinternal@rndc-usa.com, wmsconsultant@rndc-usa.com, WMSMSPSupport@RNDC-USA.COM", "ccEmail": "","footer":"","attachment":["link-to-alert","link-to-results","inline-table"]},"sql":"SELECT org_id, location_id, item_id, pack_uom_type_id, pack_uom_quantity FROM default_dcinventory.DCI_LOCATION_ITEM_ASSIGNMENT WHERE 1=1 AND org_id= $orgId AND pack_uom_type_id is NOT NULL;"}'</t>
+  </si>
+  <si>
+    <t>(unnamed, no payload entry in warehouselocationdetail)</t>
   </si>
 </sst>
 </file>
@@ -3145,34 +3145,34 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="B1" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="C1" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="D1" t="s">
         <v>6</v>
       </c>
       <c r="E1" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="F1" t="s">
         <v>122</v>
       </c>
       <c r="G1" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="H1" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="I1" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="J1" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -3192,16 +3192,16 @@
         <v>31</v>
       </c>
       <c r="F2" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="G2" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H2" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I2" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J2" s="16">
         <v>46084.901155428241</v>
@@ -3227,13 +3227,13 @@
         <v>123</v>
       </c>
       <c r="G3" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H3" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I3" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J3" s="16">
         <v>46084.901155428241</v>
@@ -3259,13 +3259,13 @@
         <v>123</v>
       </c>
       <c r="G4" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H4" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I4" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J4" s="16">
         <v>46084.901155428241</v>
@@ -3291,13 +3291,13 @@
         <v>123</v>
       </c>
       <c r="G5" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H5" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I5" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J5" s="16">
         <v>46084.901155428241</v>
@@ -3323,13 +3323,13 @@
         <v>123</v>
       </c>
       <c r="G6" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H6" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I6" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J6" s="16">
         <v>46084.901155428241</v>
@@ -3355,13 +3355,13 @@
         <v>123</v>
       </c>
       <c r="G7" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H7" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I7" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J7" s="16">
         <v>46084.901155428241</v>
@@ -3387,13 +3387,13 @@
         <v>123</v>
       </c>
       <c r="G8" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H8" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I8" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J8" s="16">
         <v>46084.901155428241</v>
@@ -3419,13 +3419,13 @@
         <v>123</v>
       </c>
       <c r="G9" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H9" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I9" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J9" s="16">
         <v>46084.901155428241</v>
@@ -3451,13 +3451,13 @@
         <v>123</v>
       </c>
       <c r="G10" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H10" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I10" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J10" s="16">
         <v>46084.901155428241</v>
@@ -3480,16 +3480,16 @@
         <v>31</v>
       </c>
       <c r="F11" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="G11" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H11" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I11" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J11" s="16">
         <v>46084.901155428241</v>
@@ -3515,13 +3515,13 @@
         <v>123</v>
       </c>
       <c r="G12" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H12" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I12" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J12" s="16">
         <v>46084.901155428241</v>
@@ -3547,13 +3547,13 @@
         <v>123</v>
       </c>
       <c r="G13" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H13" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I13" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J13" s="16">
         <v>46084.901155428241</v>
@@ -3579,13 +3579,13 @@
         <v>123</v>
       </c>
       <c r="G14" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H14" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I14" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J14" s="16">
         <v>46084.901155428241</v>
@@ -3608,16 +3608,16 @@
         <v>31</v>
       </c>
       <c r="F15" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="G15" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H15" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I15" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J15" s="16">
         <v>46084.901155428241</v>
@@ -3643,13 +3643,13 @@
         <v>123</v>
       </c>
       <c r="G16" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H16" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I16" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J16" s="16">
         <v>46084.901155428241</v>
@@ -3675,13 +3675,13 @@
         <v>123</v>
       </c>
       <c r="G17" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H17" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I17" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J17" s="16">
         <v>46084.901155428241</v>
@@ -3707,13 +3707,13 @@
         <v>123</v>
       </c>
       <c r="G18" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H18" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I18" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J18" s="16">
         <v>46084.901155428241</v>
@@ -3739,13 +3739,13 @@
         <v>123</v>
       </c>
       <c r="G19" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H19" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I19" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J19" s="16">
         <v>46084.901155428241</v>
@@ -3771,13 +3771,13 @@
         <v>123</v>
       </c>
       <c r="G20" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H20" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I20" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J20" s="16">
         <v>46084.901155428241</v>
@@ -3803,13 +3803,13 @@
         <v>123</v>
       </c>
       <c r="G21" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H21" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I21" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J21" s="16">
         <v>46084.901155428241</v>
@@ -3835,13 +3835,13 @@
         <v>123</v>
       </c>
       <c r="G22" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H22" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I22" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J22" s="16">
         <v>46084.901155428241</v>
@@ -3867,13 +3867,13 @@
         <v>123</v>
       </c>
       <c r="G23" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H23" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I23" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J23" s="16">
         <v>46084.901155428241</v>
@@ -3899,13 +3899,13 @@
         <v>123</v>
       </c>
       <c r="G24" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H24" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I24" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J24" s="16">
         <v>46084.901155428241</v>
@@ -3931,13 +3931,13 @@
         <v>123</v>
       </c>
       <c r="G25" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H25" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I25" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J25" s="16">
         <v>46084.901155428241</v>
@@ -3960,16 +3960,16 @@
         <v>31</v>
       </c>
       <c r="F26" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="G26" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H26" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I26" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J26" s="16">
         <v>46084.901155428241</v>
@@ -3995,13 +3995,13 @@
         <v>123</v>
       </c>
       <c r="G27" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H27" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I27" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J27" s="16">
         <v>46084.901155428241</v>
@@ -4027,13 +4027,13 @@
         <v>123</v>
       </c>
       <c r="G28" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H28" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I28" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J28" s="16">
         <v>46084.901155428241</v>
@@ -4059,13 +4059,13 @@
         <v>123</v>
       </c>
       <c r="G29" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H29" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I29" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J29" s="16">
         <v>46084.901155428241</v>
@@ -4088,16 +4088,16 @@
         <v>31</v>
       </c>
       <c r="F30" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="G30" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H30" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I30" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J30" s="16">
         <v>46084.901155428241</v>
@@ -4123,13 +4123,13 @@
         <v>123</v>
       </c>
       <c r="G31" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H31" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I31" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J31" s="16">
         <v>46084.901155428241</v>
@@ -4155,13 +4155,13 @@
         <v>123</v>
       </c>
       <c r="G32" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H32" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I32" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J32" s="16">
         <v>46084.901155428241</v>
@@ -4187,13 +4187,13 @@
         <v>123</v>
       </c>
       <c r="G33" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H33" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I33" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J33" s="16">
         <v>46084.901155428241</v>
@@ -4219,13 +4219,13 @@
         <v>123</v>
       </c>
       <c r="G34" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H34" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I34" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J34" s="16">
         <v>46084.901155428241</v>
@@ -4251,13 +4251,13 @@
         <v>123</v>
       </c>
       <c r="G35" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H35" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I35" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J35" s="16">
         <v>46084.901155428241</v>
@@ -4283,13 +4283,13 @@
         <v>123</v>
       </c>
       <c r="G36" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H36" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I36" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J36" s="16">
         <v>46084.901155428241</v>
@@ -4315,13 +4315,13 @@
         <v>123</v>
       </c>
       <c r="G37" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H37" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I37" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J37" s="16">
         <v>46084.901155428241</v>
@@ -4347,13 +4347,13 @@
         <v>123</v>
       </c>
       <c r="G38" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H38" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I38" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J38" s="16">
         <v>46084.901155428241</v>
@@ -4379,13 +4379,13 @@
         <v>123</v>
       </c>
       <c r="G39" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H39" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I39" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J39" s="16">
         <v>46084.901155428241</v>
@@ -4411,13 +4411,13 @@
         <v>123</v>
       </c>
       <c r="G40" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H40" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I40" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J40" s="16">
         <v>46084.901155428241</v>
@@ -4443,13 +4443,13 @@
         <v>123</v>
       </c>
       <c r="G41" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H41" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I41" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J41" s="16">
         <v>46084.901155428241</v>
@@ -4472,16 +4472,16 @@
         <v>31</v>
       </c>
       <c r="F42" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="G42" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H42" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I42" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J42" s="16">
         <v>46084.901155428241</v>
@@ -4507,13 +4507,13 @@
         <v>123</v>
       </c>
       <c r="G43" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H43" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I43" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J43" s="16">
         <v>46084.901155428241</v>
@@ -4539,13 +4539,13 @@
         <v>123</v>
       </c>
       <c r="G44" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="H44" s="16">
         <v>46084.901155428241</v>
       </c>
       <c r="I44" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="J44" s="16">
         <v>46084.901155428241</v>
@@ -4558,6 +4558,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A63BE434-9ED0-E94E-BE21-7A21279D6729}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -4600,7 +4601,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="102" x14ac:dyDescent="0.2">
       <c r="A2" t="b">
         <v>0</v>
       </c>
@@ -4620,7 +4621,7 @@
         <v>31</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>174</v>
@@ -4636,7 +4637,7 @@
       </c>
       <c r="L2" s="14"/>
     </row>
-    <row r="3" spans="1:12" ht="119" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="102" x14ac:dyDescent="0.2">
       <c r="A3" t="b">
         <v>0</v>
       </c>
@@ -4656,7 +4657,7 @@
         <v>31</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>174</v>
@@ -4671,7 +4672,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="102" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="b">
         <v>1</v>
       </c>
@@ -4691,7 +4692,7 @@
         <v>31</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>174</v>
@@ -4707,7 +4708,7 @@
       </c>
       <c r="L4" s="3"/>
     </row>
-    <row r="5" spans="1:12" ht="102" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="b">
         <v>1</v>
       </c>
@@ -4727,7 +4728,7 @@
         <v>31</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>174</v>
@@ -4742,7 +4743,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="85" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="b">
         <v>1</v>
       </c>
@@ -4762,7 +4763,7 @@
         <v>31</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>174</v>
@@ -4777,7 +4778,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="102" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="b">
         <v>1</v>
       </c>
@@ -4797,7 +4798,7 @@
         <v>31</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>222</v>
+        <v>239</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>174</v>
@@ -4812,7 +4813,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="102" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" t="b">
         <v>0</v>
       </c>
@@ -4832,7 +4833,7 @@
         <v>31</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>174</v>
@@ -4847,7 +4848,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="102" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" t="b">
         <v>0</v>
       </c>
@@ -4867,7 +4868,7 @@
         <v>31</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>174</v>
@@ -4901,8 +4902,8 @@
       <c r="F10" s="3">
         <v>31</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>221</v>
+      <c r="G10" s="15" t="s">
+        <v>244</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>174</v>
@@ -4917,7 +4918,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="85" x14ac:dyDescent="0.2">
       <c r="A11" t="b">
         <v>0</v>
       </c>
@@ -4936,8 +4937,8 @@
       <c r="F11" s="3">
         <v>31</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>221</v>
+      <c r="G11" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>174</v>
@@ -4952,7 +4953,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="85" x14ac:dyDescent="0.2">
       <c r="A12" t="b">
         <v>0</v>
       </c>
@@ -4971,8 +4972,8 @@
       <c r="F12" s="3">
         <v>31</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>221</v>
+      <c r="G12" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>174</v>
@@ -4987,7 +4988,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" ht="85" x14ac:dyDescent="0.2">
       <c r="A13" t="b">
         <v>0</v>
       </c>
@@ -5006,8 +5007,8 @@
       <c r="F13" s="3">
         <v>31</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>221</v>
+      <c r="G13" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>174</v>
@@ -5022,7 +5023,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" ht="85" x14ac:dyDescent="0.2">
       <c r="A14" t="b">
         <v>0</v>
       </c>
@@ -5041,8 +5042,8 @@
       <c r="F14" s="3">
         <v>31</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>221</v>
+      <c r="G14" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>174</v>
@@ -5057,7 +5058,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ht="85" x14ac:dyDescent="0.2">
       <c r="A15" t="b">
         <v>0</v>
       </c>
@@ -5076,8 +5077,8 @@
       <c r="F15" s="3">
         <v>31</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>221</v>
+      <c r="G15" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>174</v>
@@ -5092,7 +5093,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ht="85" x14ac:dyDescent="0.2">
       <c r="A16" t="b">
         <v>0</v>
       </c>
@@ -5111,8 +5112,8 @@
       <c r="F16" s="3">
         <v>31</v>
       </c>
-      <c r="G16" s="3" t="s">
-        <v>221</v>
+      <c r="G16" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>174</v>
@@ -5127,7 +5128,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A17" t="b">
         <v>0</v>
       </c>
@@ -5146,8 +5147,8 @@
       <c r="F17" s="3">
         <v>31</v>
       </c>
-      <c r="G17" s="3" t="s">
-        <v>221</v>
+      <c r="G17" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>174</v>
@@ -5162,7 +5163,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A18" t="b">
         <v>0</v>
       </c>
@@ -5181,8 +5182,8 @@
       <c r="F18" s="3">
         <v>31</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>221</v>
+      <c r="G18" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>174</v>
@@ -5197,7 +5198,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A19" t="b">
         <v>0</v>
       </c>
@@ -5216,8 +5217,8 @@
       <c r="F19" s="3">
         <v>31</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>221</v>
+      <c r="G19" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>174</v>
@@ -5232,7 +5233,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A20" t="b">
         <v>0</v>
       </c>
@@ -5251,8 +5252,8 @@
       <c r="F20" s="3">
         <v>31</v>
       </c>
-      <c r="G20" s="3" t="s">
-        <v>221</v>
+      <c r="G20" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>174</v>
@@ -5267,7 +5268,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A21" t="b">
         <v>0</v>
       </c>
@@ -5286,8 +5287,8 @@
       <c r="F21" s="3">
         <v>31</v>
       </c>
-      <c r="G21" s="3" t="s">
-        <v>221</v>
+      <c r="G21" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>174</v>
@@ -5302,7 +5303,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A22" t="b">
         <v>0</v>
       </c>
@@ -5321,8 +5322,8 @@
       <c r="F22" s="3">
         <v>31</v>
       </c>
-      <c r="G22" s="3" t="s">
-        <v>221</v>
+      <c r="G22" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>174</v>
@@ -5337,7 +5338,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A23" t="b">
         <v>0</v>
       </c>
@@ -5356,8 +5357,8 @@
       <c r="F23" s="3">
         <v>31</v>
       </c>
-      <c r="G23" s="3" t="s">
-        <v>221</v>
+      <c r="G23" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>174</v>
@@ -5372,7 +5373,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A24" t="b">
         <v>0</v>
       </c>
@@ -5391,8 +5392,8 @@
       <c r="F24" s="3">
         <v>31</v>
       </c>
-      <c r="G24" s="3" t="s">
-        <v>221</v>
+      <c r="G24" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>174</v>
@@ -5407,7 +5408,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A25" t="b">
         <v>0</v>
       </c>
@@ -5426,8 +5427,8 @@
       <c r="F25" s="3">
         <v>31</v>
       </c>
-      <c r="G25" s="3" t="s">
-        <v>221</v>
+      <c r="G25" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>174</v>
@@ -5442,7 +5443,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A26" t="b">
         <v>0</v>
       </c>
@@ -5461,8 +5462,8 @@
       <c r="F26" s="3">
         <v>31</v>
       </c>
-      <c r="G26" s="3" t="s">
-        <v>221</v>
+      <c r="G26" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>174</v>
@@ -5477,7 +5478,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A27" t="b">
         <v>0</v>
       </c>
@@ -5496,8 +5497,8 @@
       <c r="F27" s="3">
         <v>31</v>
       </c>
-      <c r="G27" s="3" t="s">
-        <v>221</v>
+      <c r="G27" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>174</v>
@@ -5512,7 +5513,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A28" t="b">
         <v>0</v>
       </c>
@@ -5531,8 +5532,8 @@
       <c r="F28" s="3">
         <v>31</v>
       </c>
-      <c r="G28" s="3" t="s">
-        <v>221</v>
+      <c r="G28" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>174</v>
@@ -5547,7 +5548,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A29" t="b">
         <v>0</v>
       </c>
@@ -5566,8 +5567,8 @@
       <c r="F29" s="3">
         <v>31</v>
       </c>
-      <c r="G29" s="3" t="s">
-        <v>221</v>
+      <c r="G29" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>174</v>
@@ -5582,7 +5583,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A30" t="b">
         <v>0</v>
       </c>
@@ -5601,8 +5602,8 @@
       <c r="F30" s="3">
         <v>31</v>
       </c>
-      <c r="G30" s="3" t="s">
-        <v>221</v>
+      <c r="G30" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>174</v>
@@ -5636,8 +5637,8 @@
       <c r="F31" s="3">
         <v>31</v>
       </c>
-      <c r="G31" s="3" t="s">
-        <v>221</v>
+      <c r="G31" s="15" t="s">
+        <v>244</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>174</v>
@@ -5652,7 +5653,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A32" t="b">
         <v>0</v>
       </c>
@@ -5671,8 +5672,8 @@
       <c r="F32" s="3">
         <v>31</v>
       </c>
-      <c r="G32" s="3" t="s">
-        <v>221</v>
+      <c r="G32" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>174</v>
@@ -5687,7 +5688,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A33" t="b">
         <v>0</v>
       </c>
@@ -5706,8 +5707,8 @@
       <c r="F33" s="3">
         <v>31</v>
       </c>
-      <c r="G33" s="3" t="s">
-        <v>221</v>
+      <c r="G33" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>174</v>
@@ -5722,7 +5723,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A34" t="b">
         <v>0</v>
       </c>
@@ -5741,8 +5742,8 @@
       <c r="F34" s="3">
         <v>31</v>
       </c>
-      <c r="G34" s="3" t="s">
-        <v>221</v>
+      <c r="G34" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>174</v>
@@ -5757,7 +5758,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A35" t="b">
         <v>0</v>
       </c>
@@ -5776,8 +5777,8 @@
       <c r="F35" s="3">
         <v>31</v>
       </c>
-      <c r="G35" s="3" t="s">
-        <v>221</v>
+      <c r="G35" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>174</v>
@@ -5792,7 +5793,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A36" t="b">
         <v>0</v>
       </c>
@@ -5811,8 +5812,8 @@
       <c r="F36" s="3">
         <v>31</v>
       </c>
-      <c r="G36" s="3" t="s">
-        <v>221</v>
+      <c r="G36" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>174</v>
@@ -5827,7 +5828,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A37" t="b">
         <v>0</v>
       </c>
@@ -5846,8 +5847,8 @@
       <c r="F37" s="3">
         <v>31</v>
       </c>
-      <c r="G37" s="3" t="s">
-        <v>221</v>
+      <c r="G37" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>174</v>
@@ -5862,7 +5863,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A38" t="b">
         <v>0</v>
       </c>
@@ -5881,8 +5882,8 @@
       <c r="F38" s="3">
         <v>31</v>
       </c>
-      <c r="G38" s="3" t="s">
-        <v>221</v>
+      <c r="G38" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>174</v>
@@ -5916,8 +5917,8 @@
       <c r="F39" s="3">
         <v>31</v>
       </c>
-      <c r="G39" s="3" t="s">
-        <v>221</v>
+      <c r="G39" s="15" t="s">
+        <v>244</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>174</v>
@@ -5951,8 +5952,8 @@
       <c r="F40" s="3">
         <v>31</v>
       </c>
-      <c r="G40" s="3" t="s">
-        <v>221</v>
+      <c r="G40" s="15" t="s">
+        <v>244</v>
       </c>
       <c r="H40" s="3" t="s">
         <v>174</v>
@@ -5967,7 +5968,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A41" t="b">
         <v>0</v>
       </c>
@@ -5986,8 +5987,8 @@
       <c r="F41" s="3">
         <v>31</v>
       </c>
-      <c r="G41" s="3" t="s">
-        <v>221</v>
+      <c r="G41" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>174</v>
@@ -6002,7 +6003,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A42" t="b">
         <v>0</v>
       </c>
@@ -6021,8 +6022,8 @@
       <c r="F42" s="3">
         <v>31</v>
       </c>
-      <c r="G42" s="3" t="s">
-        <v>221</v>
+      <c r="G42" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>174</v>
@@ -6037,7 +6038,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A43" t="b">
         <v>0</v>
       </c>
@@ -6056,8 +6057,8 @@
       <c r="F43" s="3">
         <v>31</v>
       </c>
-      <c r="G43" s="3" t="s">
-        <v>221</v>
+      <c r="G43" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>174</v>
@@ -6072,7 +6073,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" ht="85" x14ac:dyDescent="0.2">
       <c r="A44" t="b">
         <v>0</v>
       </c>
@@ -6091,8 +6092,8 @@
       <c r="F44" s="3">
         <v>31</v>
       </c>
-      <c r="G44" s="3" t="s">
-        <v>221</v>
+      <c r="G44" s="15" t="s">
+        <v>243</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>174</v>
@@ -6107,12 +6108,12 @@
         <v>175</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="C45" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="C46" s="3">
         <v>1</v>
       </c>
@@ -6120,7 +6121,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="C47" s="3">
         <v>40</v>
       </c>
@@ -6129,7 +6130,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K47" xr:uid="{A63BE434-9ED0-E94E-BE21-7A21279D6729}"/>
+  <autoFilter ref="A1:K47" xr:uid="{A63BE434-9ED0-E94E-BE21-7A21279D6729}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="FALSE"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>